<commit_message>
updated docs in verif. and superization.py
</commit_message>
<xml_diff>
--- a/verification_burde/explicit_rep_LSS_burde.xlsx
+++ b/verification_burde/explicit_rep_LSS_burde.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/josemarialoza/capstone/verification_burde/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DF13E56-2ADD-F14D-B146-ADAF26C43EDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7158992D-DA84-1541-8F3B-1504EA4B3653}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="840" windowWidth="27640" windowHeight="16720" activeTab="1" xr2:uid="{963206F1-EDEA-1A45-9EF5-B0667A40C611}"/>
+    <workbookView xWindow="1080" yWindow="840" windowWidth="27640" windowHeight="16720" xr2:uid="{963206F1-EDEA-1A45-9EF5-B0667A40C611}"/>
   </bookViews>
   <sheets>
     <sheet name="Explicit Reps." sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="138">
   <si>
     <t>LSS 1</t>
   </si>
@@ -418,6 +418,60 @@
   </si>
   <si>
     <t>X ~ Y</t>
+  </si>
+  <si>
+    <t>LSS 3</t>
+  </si>
+  <si>
+    <t>LSS 4</t>
+  </si>
+  <si>
+    <t>lambda_E(F) = 0</t>
+  </si>
+  <si>
+    <t>lambda_E(H) = -E</t>
+  </si>
+  <si>
+    <t>lambda_F(E) = -H</t>
+  </si>
+  <si>
+    <t>lambda_F(F) = E - H</t>
+  </si>
+  <si>
+    <t>lambda_F(H) = E - F</t>
+  </si>
+  <si>
+    <t>lambda_H(E) = E</t>
+  </si>
+  <si>
+    <t>lambda_H(F) = E</t>
+  </si>
+  <si>
+    <t>lambda_H(H) = -H</t>
+  </si>
+  <si>
+    <t>lambda_E(F) = (b-1)H</t>
+  </si>
+  <si>
+    <t>lambda_E(H) = bE</t>
+  </si>
+  <si>
+    <t>lambda_F(E) = (b + 1)H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lambda_F(F) = E </t>
+  </si>
+  <si>
+    <t>lambda_F(H) = bF</t>
+  </si>
+  <si>
+    <t>lambda_H(E) = (b - 1)E</t>
+  </si>
+  <si>
+    <t>lambda_H(F) = (b + 1)F</t>
+  </si>
+  <si>
+    <t>lambda_H(H) = bH</t>
   </si>
 </sst>
 </file>
@@ -453,7 +507,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -493,6 +547,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -561,7 +627,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -573,22 +639,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -601,6 +667,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -937,7 +1009,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B836528E-83CA-3640-9E8D-70989B61B880}">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="12.1640625" customWidth="1"/>
@@ -945,159 +1017,347 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
+      <c r="A1" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="5"/>
+      <c r="C2" s="6"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5" t="s">
+      <c r="A3" s="6"/>
+      <c r="B3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="5"/>
+      <c r="C3" s="6"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5" t="s">
+      <c r="A4" s="6"/>
+      <c r="B4" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="5"/>
+      <c r="C4" s="6"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="6"/>
+      <c r="C5" s="5"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="6"/>
-      <c r="B6" s="6" t="s">
+      <c r="A6" s="5"/>
+      <c r="B6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="6"/>
+      <c r="C6" s="5"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="6"/>
-      <c r="B7" s="6" t="s">
+      <c r="A7" s="5"/>
+      <c r="B7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="6"/>
+      <c r="C7" s="5"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="10"/>
+      <c r="C8" s="8"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="9"/>
-      <c r="B9" s="10" t="s">
+      <c r="A9" s="7"/>
+      <c r="B9" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="10"/>
+      <c r="C9" s="8"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="9"/>
-      <c r="B10" s="10" t="s">
+      <c r="A10" s="7"/>
+      <c r="B10" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="10"/>
+      <c r="C10" s="8"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="5"/>
+      <c r="C12" s="6"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5" t="s">
+      <c r="A13" s="6"/>
+      <c r="B13" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="C13" s="5"/>
+      <c r="C13" s="6"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5" t="s">
+      <c r="A14" s="6"/>
+      <c r="B14" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C14" s="5"/>
+      <c r="C14" s="6"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="C15" s="6"/>
+      <c r="C15" s="5"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" s="6"/>
-      <c r="B16" s="6" t="s">
+      <c r="A16" s="5"/>
+      <c r="B16" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="6"/>
+      <c r="C16" s="5"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" s="6"/>
-      <c r="B17" s="6" t="s">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C17" s="6"/>
+      <c r="C17" s="5"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="9" t="s">
+      <c r="A18" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="C18" s="10"/>
+      <c r="C18" s="8"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" s="9"/>
-      <c r="B19" s="10" t="s">
+      <c r="A19" s="7"/>
+      <c r="B19" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="C19" s="10"/>
+      <c r="C19" s="8"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" s="9"/>
-      <c r="B20" s="10" t="s">
+      <c r="A20" s="7"/>
+      <c r="B20" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="C20" s="10"/>
+      <c r="C20" s="8"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="B21" s="15"/>
+      <c r="C21" s="15"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C22" s="6"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" s="6"/>
+      <c r="B23" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C23" s="6"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" s="6"/>
+      <c r="B24" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="C24" s="6"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C25" s="5"/>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" s="5"/>
+      <c r="B26" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="C26" s="5"/>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" s="5"/>
+      <c r="B27" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="C27" s="5"/>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="C28" s="8"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" s="7"/>
+      <c r="B29" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="C29" s="8"/>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" s="7"/>
+      <c r="B30" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="C30" s="8"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="B31" s="16"/>
+      <c r="C31" s="16"/>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C32" s="6"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" s="6"/>
+      <c r="B33" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="C33" s="6"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" s="6"/>
+      <c r="B34" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="C34" s="6"/>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="C35" s="5"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" s="5"/>
+      <c r="B36" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C36" s="5"/>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" s="5"/>
+      <c r="B37" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="C37" s="5"/>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="C38" s="8"/>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" s="7"/>
+      <c r="B39" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="C39" s="8"/>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" s="7"/>
+      <c r="B40" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="C40" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="26">
+  <mergeCells count="52">
+    <mergeCell ref="A35:A37"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="A38:A40"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A32:A34"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="A25:A27"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="A28:A30"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B10:C10"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="A12:A14"/>
     <mergeCell ref="A15:A17"/>
@@ -1114,16 +1374,6 @@
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="A5:A7"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B10:C10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>